<commit_message>
Rebuild final RC Assets list from pushed CSV source
</commit_message>
<xml_diff>
--- a/final_lists/rc_assets_final_scanned_list/output_excel/rc_assets_removed_red_strikethrough.xlsx
+++ b/final_lists/rc_assets_final_scanned_list/output_excel/rc_assets_removed_red_strikethrough.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Removed Red Crossed Out" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Removed Red Crossed Out'!$A$1:$S$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Removed Red Crossed Out'!$A$1:$T$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -44,7 +44,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -52,13 +52,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -426,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -443,11 +457,12 @@
     <col width="25" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
     <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="32" customWidth="1" min="18" max="18"/>
-    <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="32" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -523,32 +538,37 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>source_excel_row</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>red_indicator_detected</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>strikethrough_detected</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>crossed_out_indicator_detected</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>cleaning_action</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S1"/>
+  <autoFilter ref="A1:T1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>